<commit_message>
updated home page image and data update
</commit_message>
<xml_diff>
--- a/excels/AcademicPrograms.xlsx
+++ b/excels/AcademicPrograms.xlsx
@@ -5,11 +5,11 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\fmain\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="12150" activeTab="1"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="10350" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Mtech" sheetId="1" r:id="rId1"/>
@@ -48,9 +48,6 @@
     <t xml:space="preserve">2 years </t>
   </si>
   <si>
-    <t>5years</t>
-  </si>
-  <si>
     <t>The application form is to be submitted online, which is available at https://admissions.nitw.ac.in/ (Copy the above link and paste in the browser) All the necessary documents are to be uploaded online. The link to pay registration fee (Rs. 1000/- for GEN/ GEN-EWS/ OBC-NCL and Rs. 500/- for SC/ ST/ PwD candidates) is given in the candidate’s registered login page.</t>
   </si>
   <si>
@@ -206,9 +203,6 @@
   </si>
   <si>
     <t>https://admissions.nitw.ac.in/media/uploadsbyadmin/20260327_222139_phd_j_2026.pdf</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sustainable Transportation, Traffic Safety, Travel Behaviour,Land Use Transport Planning ,Low Volume Roads, Public Transportation, Road Safety, Sustainable Transport, Transit Oriented Development, Transport Economics, Travel Demand Modelling, Urban Transportation Planning, Asphalt pavement analysis, Design and evaluation , Characterization of asphalt binders and mixtures, Quantification of roadway and railway traffic noise, Forensic Investigations of Pavement Failures, Low Volume Road Engineering, New and Innovative Marginal Materials in Low Volume Roads, Pavement Management System, Pavement Material's, Recylcing of Pavement Materials, Subgrade Stabilization and Geosynthetics i Rural Roads, Sustainable Pavement Maintenance Strategies , Traffic emission and level of service, Traffic Flow Modeling, Highway Capacity, Geometric Design, Pavement Forensics, Pavement Management Systems, Pavement Recycling , Rheology of Bituminous binders and Mixes, Congestion Management and ITS, Crowd Dynamic and Emergency Evacuation Planning, Highway Capacity Analysis, Road User Behaviour Study and Safety Enhancement , Safety Analysis of Vehicular and Pedestrian Interactions. </t>
   </si>
   <si>
     <t>Assistant Professor, Associate Professor, Research Faculty ,Transportation Researcher, Senior Scientist, R&amp;D Specialist,Transportation Officer, Highway Engineer, Technical Advisor, Pavement Research Engineer, Traffic Simulation Expert</t>
@@ -667,6 +661,95 @@
         <scheme val="minor"/>
       </rPr>
       <t>) Executive PhD Program : Open for all working professionals. M.Tech. students from NIT Warangal can also enroll in the Executive Ph.D programs in their respective disciplines after completing their degree. The eligibility criteria are the same as those for the regular Ph.D program (under the self-finance category). These scholars must complete 4 Online Certifications (such as NPTEL), as recommended by the DSC, within one year. No minimum work experience is required for admissions. Scholars admitted under Executive Ph.D. are exempted from the minimum residential requirement.</t>
+    </r>
+  </si>
+  <si>
+    <t>Minimum Duration 5years</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Pavements                              </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">:  Asphalt pavement analysis, design and evaluation, Characterization of asphalt binders and mixtures, Forensic Investigations of Pavement Failures, Low Volume Road Engineering, Low Volume Roads, New and Innovative Marginal Materials in Low Volume Roads, Pavement Management System, Pavement Materials, Pavement Recycling, Recycling of Pavement Materials, Rheology of Bituminous Binders and Mixes, Subgrade Stabilization and Geosynthetics in Rural Roads, Sustainable Pavement Maintenance Strategies, Pavement Forensics.                                                                                                                                                                                                                                                                      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Traffic Engineering              :</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  Traffic Safety,  Road Safety, Traffic Flow Modeling, Highway Capacity, Highway Capacity Analysis, Geometric Design, Traffic emission and Level of Service, Congestion Management and Intelligent Transportation Systems (ITS), Road User Behaviour Study and Safety Enhancement, Safety Analysis of Vehicular and Pedestrian Interactions, Quantification of Roadway and Railway Traffic Noise                                                                                                                                                                                                                                                                    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Urban Transport Planning  :  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Sustainable Transportation,Travel Behaviour, Land Use Transport Planning, Public Transportation, Transit Oriented Development (TOD),  Transport Economics, Travel Demand Modelling ,Urban Transportation Planning, Crowd Dynamics and Emergency Evacuation Planning                                                                                                                                                      </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">                                                                                                                                                                           </t>
     </r>
   </si>
 </sst>
@@ -1044,10 +1127,10 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
         <v>14</v>
-      </c>
-      <c r="B2" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -1055,15 +1138,15 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="375" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1071,7 +1154,7 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1079,7 +1162,7 @@
         <v>4</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1087,15 +1170,15 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -1113,7 +1196,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.5703125" customWidth="1"/>
-    <col min="2" max="2" width="104.85546875" customWidth="1"/>
+    <col min="2" max="2" width="159.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1121,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>7</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="181.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1129,15 +1212,15 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" ht="135" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>23</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" ht="165" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1145,7 +1228,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1153,7 +1236,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
@@ -1161,15 +1244,15 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
academic programs duration update
</commit_message>
<xml_diff>
--- a/excels/AcademicPrograms.xlsx
+++ b/excels/AcademicPrograms.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\CED TD-11\Downloads\mainnn\NITW-Transportation-Division-main\excels\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\code\nitw\NITW-Transportation-Division\excels\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F6ADFFF-22D3-49C7-8BC7-EB2FFAA7FB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14370" windowHeight="10350" activeTab="1"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mtech" sheetId="1" r:id="rId1"/>
@@ -664,9 +665,6 @@
     </r>
   </si>
   <si>
-    <t>Minimum Duration 5years</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -751,12 +749,15 @@
       </rPr>
       <t xml:space="preserve">                                                                                                                                                                           </t>
     </r>
+  </si>
+  <si>
+    <t>Minimum Duration of 3years(FullTime) or 5years (PartTime)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1109,7 +1110,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1183,15 +1184,15 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B6" r:id="rId1"/>
-    <hyperlink ref="B8" r:id="rId2"/>
+    <hyperlink ref="B6" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
+    <hyperlink ref="B8" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1204,7 +1205,7 @@
         <v>0</v>
       </c>
       <c r="B1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="181.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1220,7 +1221,7 @@
         <v>8</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1257,9 +1258,9 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B7" r:id="rId1"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://admissions.nitw.ac.in/media/uploadsbyadmin/20260327_222139_phd_j_2026.pdf"/>
-    <hyperlink ref="B5" r:id="rId3"/>
+    <hyperlink ref="B7" r:id="rId1" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://admissions.nitw.ac.in/media/uploadsbyadmin/20260327_222139_phd_j_2026.pdf" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{00000000-0004-0000-0100-000002000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>